<commit_message>
Se ajusta el manual de usuario y las pruebas usabilidad
</commit_message>
<xml_diff>
--- a/docs/pruebas_usabilidad_ieee29119-11.xlsx
+++ b/docs/pruebas_usabilidad_ieee29119-11.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13392"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13390"/>
   </bookViews>
   <sheets>
     <sheet name="plantilla_registro_pruebas_usab" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="97">
   <si>
     <t>ID Registro</t>
   </si>
@@ -153,19 +153,19 @@
     <t>USAB-004</t>
   </si>
   <si>
-    <t>Trabajos (Wizard)</t>
+    <t>Trabajos (Wizard + filtros de archivo)</t>
   </si>
   <si>
     <t>Creacion de respaldo</t>
   </si>
   <si>
-    <t>Crear trabajo completo con filtros destino programacion y scripts</t>
-  </si>
-  <si>
-    <t>Flujo entendible, sin retrocesos innecesarios, &lt;= 5 min</t>
-  </si>
-  <si>
-    <t>Carpeta origen + destino + reglas</t>
+    <t>Crear trabajo completo con exclusiones y filtros por tamano/creacion/actualizacion</t>
+  </si>
+  <si>
+    <t>Flujo entendible, sin retrocesos innecesarios, &lt;= 6 min; usuario comprende los filtros y corrige validaciones si hay rangos invalidos</t>
+  </si>
+  <si>
+    <t>Carpeta origen + destino + filtros por metadatos + programacion + scripts</t>
   </si>
   <si>
     <t>Trabajo guardado correctamente</t>
@@ -253,128 +253,73 @@
   </si>
   <si>
     <t>Trabajo se ejecuta automaticamente segun agenda y registra resultados</t>
+  </si>
+  <si>
+    <t>USAB-010</t>
+  </si>
+  <si>
+    <t>Filtros de archivo (tamano)</t>
+  </si>
+  <si>
+    <t>Creacion de trabajo con filtros</t>
+  </si>
+  <si>
+    <t>Configurar tamano minimo y maximo en wizard</t>
+  </si>
+  <si>
+    <t>Usuario identifica unidad MiB, entiende campos opcionales y completa sin ayuda en &lt;= 2 min</t>
+  </si>
+  <si>
+    <t>Tamano minimo=1 MiB, tamano maximo=10 MiB</t>
+  </si>
+  <si>
+    <t>Trabajo guarda filtros correctamente y no muestra errores de validacion</t>
+  </si>
+  <si>
+    <t>USAB-011</t>
+  </si>
+  <si>
+    <t>Filtros de archivo (fechas)</t>
+  </si>
+  <si>
+    <t>Configurar rango de creacion y actualizacion</t>
+  </si>
+  <si>
+    <t>Usuario comprende formato fecha/hora y mensajes cuando desde &gt; hasta</t>
+  </si>
+  <si>
+    <t>Creacion desde/hasta y actualizacion desde/hasta</t>
+  </si>
+  <si>
+    <t>Sistema bloquea rangos invalidos y permite guardar rangos validos</t>
+  </si>
+  <si>
+    <t>Ejecucion con filtros activos</t>
+  </si>
+  <si>
+    <t>Ejecutar manualmente trabajo con filtros y revisar reporte</t>
+  </si>
+  <si>
+    <t>Usuario interpreta el resultado de 0 archivos o N archivos copiados sin confusion</t>
+  </si>
+  <si>
+    <t>Trabajo con filtros restrictivos y luego filtros ampliados</t>
+  </si>
+  <si>
+    <t>Resultado y mensaje final son claros para explicar efecto de filtros</t>
+  </si>
+  <si>
+    <t>USAB-009</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -388,13 +333,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color theme="1"/>
@@ -403,188 +341,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -592,206 +357,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="42">
-    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1069,32 +645,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:U14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="54.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="97.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="60.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="27.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="31.77734375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="54.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="97.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="60.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.6328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="20.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1159,7 +735,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1188,7 +764,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -1217,7 +793,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -1246,7 +822,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1275,7 +851,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -1304,7 +880,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -1333,7 +909,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>64</v>
       </c>
@@ -1362,7 +938,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -1391,8 +967,98 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C11">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G11" t="s">
+        <v>81</v>
+      </c>
+      <c r="H11" t="s">
+        <v>82</v>
+      </c>
+      <c r="I11" t="s">
+        <v>83</v>
+      </c>
+      <c r="J11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D12" t="s">
+        <v>86</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>80</v>
+      </c>
+      <c r="G12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H12" t="s">
+        <v>88</v>
+      </c>
+      <c r="I12" t="s">
+        <v>89</v>
+      </c>
+      <c r="J12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D13" t="s">
+        <v>91</v>
+      </c>
+      <c r="E13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" t="s">
+        <v>93</v>
+      </c>
+      <c r="I13" t="s">
+        <v>94</v>
+      </c>
+      <c r="J13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A14" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Se modifica la informacion de la seccion scriptl, el manual de usuario y se adjutan datos de la prueba de usabilidad
</commit_message>
<xml_diff>
--- a/docs/pruebas_usabilidad_ieee29119-11.xlsx
+++ b/docs/pruebas_usabilidad_ieee29119-11.xlsx
@@ -9,17 +9,19 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13390"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13392" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="plantilla_registro_pruebas_usab" sheetId="1" r:id="rId1"/>
+    <sheet name="Cesar Parra" sheetId="2" r:id="rId2"/>
+    <sheet name="Nicolas Bermudez" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="144">
   <si>
     <t>ID Registro</t>
   </si>
@@ -310,6 +312,147 @@
   </si>
   <si>
     <t>USAB-009</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>1 SEG</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>NINGUNO</t>
+  </si>
+  <si>
+    <t>NINGUNA</t>
+  </si>
+  <si>
+    <t>38 SEG</t>
+  </si>
+  <si>
+    <t>30 SEG</t>
+  </si>
+  <si>
+    <t>60 SEG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UN ERROR </t>
+  </si>
+  <si>
+    <t>FALLA</t>
+  </si>
+  <si>
+    <t>90 SEG</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>SE DETECTO EL ERROR AL NO COPIAR LA INFORMACION EN EL DESTINO, DEBIDO A QUE SE CONFIGURO MAL EL DESTINO.</t>
+  </si>
+  <si>
+    <t>MEDIA</t>
+  </si>
+  <si>
+    <t>MEJORAR LA DOCUMENTAC ION</t>
+  </si>
+  <si>
+    <t>40 SEG</t>
+  </si>
+  <si>
+    <t>CESAR P</t>
+  </si>
+  <si>
+    <t>Accedi</t>
+  </si>
+  <si>
+    <t>1seg</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Ninguno</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Nicolas Bermudez</t>
+  </si>
+  <si>
+    <t>Pude crearlo</t>
+  </si>
+  <si>
+    <t>3 min</t>
+  </si>
+  <si>
+    <t>Si</t>
+  </si>
+  <si>
+    <t>Ninguno/ pero el nombre del bucket deja pensantivo si es el full o solo el normal</t>
+  </si>
+  <si>
+    <t>BAJA</t>
+  </si>
+  <si>
+    <t>Mejorar el comentario del hallazgo</t>
+  </si>
+  <si>
+    <t>No pude crearlo</t>
+  </si>
+  <si>
+    <t>Fallo</t>
+  </si>
+  <si>
+    <t>2 min</t>
+  </si>
+  <si>
+    <t>No se pudo crear el script dificultad en saber de como se debe crear</t>
+  </si>
+  <si>
+    <t>Alta</t>
+  </si>
+  <si>
+    <t>Trabajos (Wizard)</t>
+  </si>
+  <si>
+    <t>Crear trabajo completo con filtros destino programacion y scripts</t>
+  </si>
+  <si>
+    <t>Flujo entendible, sin retrocesos innecesarios, &lt;= 5 min</t>
+  </si>
+  <si>
+    <t>Carpeta origen + destino + reglas</t>
+  </si>
+  <si>
+    <t>No se encontro problema, pero como es el computador del trabajo tiene ciertos limitantes de los permisos</t>
+  </si>
+  <si>
+    <t>Ejecutado sin problema</t>
+  </si>
+  <si>
+    <t>4 min</t>
+  </si>
+  <si>
+    <t>Solo para revisar por temas de tiempo</t>
+  </si>
+  <si>
+    <t>Poner mensaje como se esta procesando o algo para que se usario no crea que va a dar un timeout</t>
+  </si>
+  <si>
+    <t>Perfecto</t>
+  </si>
+  <si>
+    <t>Ok</t>
+  </si>
+  <si>
+    <t>Se podria mejorar colocando todas las recomendaciones que necesita porque fue ir quitando 1 tras otra hasta que me lo permitio crear, mostrar todos los errores asociados no solo 1</t>
+  </si>
+  <si>
+    <t>Baja</t>
   </si>
 </sst>
 </file>
@@ -361,10 +504,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -646,31 +792,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="54.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="97.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="60.08984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="27.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="31.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="54.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="97.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="60.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="31.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="20.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -735,7 +881,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -764,7 +910,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -793,7 +939,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -822,7 +968,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -851,7 +997,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -880,7 +1026,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -909,7 +1055,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>64</v>
       </c>
@@ -938,7 +1084,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -967,10 +1113,10 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -999,7 +1145,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>78</v>
       </c>
@@ -1028,7 +1174,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>85</v>
       </c>
@@ -1057,8 +1203,1317 @@
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:U12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" t="s">
+        <v>97</v>
+      </c>
+      <c r="L2" t="s">
+        <v>97</v>
+      </c>
+      <c r="M2" t="s">
+        <v>98</v>
+      </c>
+      <c r="N2" t="s">
+        <v>99</v>
+      </c>
+      <c r="O2" t="s">
+        <v>99</v>
+      </c>
+      <c r="P2" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>100</v>
+      </c>
+      <c r="R2" t="s">
+        <v>99</v>
+      </c>
+      <c r="S2" t="s">
+        <v>101</v>
+      </c>
+      <c r="T2" t="s">
+        <v>99</v>
+      </c>
+      <c r="U2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" t="s">
+        <v>97</v>
+      </c>
+      <c r="L3" t="s">
+        <v>97</v>
+      </c>
+      <c r="M3" t="s">
+        <v>102</v>
+      </c>
+      <c r="N3" t="s">
+        <v>99</v>
+      </c>
+      <c r="O3" t="s">
+        <v>99</v>
+      </c>
+      <c r="P3" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>100</v>
+      </c>
+      <c r="R3" t="s">
+        <v>99</v>
+      </c>
+      <c r="S3" t="s">
+        <v>101</v>
+      </c>
+      <c r="T3" t="s">
+        <v>99</v>
+      </c>
+      <c r="U3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K4" t="s">
+        <v>97</v>
+      </c>
+      <c r="L4" t="s">
+        <v>97</v>
+      </c>
+      <c r="M4" t="s">
+        <v>103</v>
+      </c>
+      <c r="N4" t="s">
+        <v>99</v>
+      </c>
+      <c r="O4" t="s">
+        <v>99</v>
+      </c>
+      <c r="P4" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>100</v>
+      </c>
+      <c r="R4" t="s">
+        <v>99</v>
+      </c>
+      <c r="S4" t="s">
+        <v>101</v>
+      </c>
+      <c r="T4" t="s">
+        <v>99</v>
+      </c>
+      <c r="U4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" t="s">
+        <v>46</v>
+      </c>
+      <c r="H5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J5" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" t="s">
+        <v>97</v>
+      </c>
+      <c r="L5" t="s">
+        <v>97</v>
+      </c>
+      <c r="M5" t="s">
+        <v>104</v>
+      </c>
+      <c r="N5" t="s">
+        <v>99</v>
+      </c>
+      <c r="O5" t="s">
+        <v>99</v>
+      </c>
+      <c r="P5" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>100</v>
+      </c>
+      <c r="R5" t="s">
+        <v>99</v>
+      </c>
+      <c r="S5" t="s">
+        <v>101</v>
+      </c>
+      <c r="T5" t="s">
+        <v>99</v>
+      </c>
+      <c r="U5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" t="s">
+        <v>55</v>
+      </c>
+      <c r="J6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K6" t="s">
+        <v>105</v>
+      </c>
+      <c r="L6" t="s">
+        <v>106</v>
+      </c>
+      <c r="M6" t="s">
+        <v>107</v>
+      </c>
+      <c r="N6" s="3">
+        <v>1</v>
+      </c>
+      <c r="O6" t="s">
+        <v>108</v>
+      </c>
+      <c r="P6" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>109</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="S6" t="s">
+        <v>111</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="U6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" t="s">
+        <v>62</v>
+      </c>
+      <c r="J7" t="s">
+        <v>63</v>
+      </c>
+      <c r="K7" t="s">
+        <v>97</v>
+      </c>
+      <c r="L7" t="s">
+        <v>97</v>
+      </c>
+      <c r="M7" t="s">
+        <v>104</v>
+      </c>
+      <c r="N7" t="s">
+        <v>99</v>
+      </c>
+      <c r="O7" t="s">
+        <v>99</v>
+      </c>
+      <c r="P7" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>100</v>
+      </c>
+      <c r="R7" t="s">
+        <v>99</v>
+      </c>
+      <c r="S7" t="s">
+        <v>101</v>
+      </c>
+      <c r="T7" t="s">
+        <v>99</v>
+      </c>
+      <c r="U7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" t="s">
+        <v>67</v>
+      </c>
+      <c r="H8" t="s">
+        <v>68</v>
+      </c>
+      <c r="I8" t="s">
+        <v>69</v>
+      </c>
+      <c r="J8" t="s">
+        <v>70</v>
+      </c>
+      <c r="K8" t="s">
+        <v>97</v>
+      </c>
+      <c r="L8" t="s">
+        <v>97</v>
+      </c>
+      <c r="M8" t="s">
+        <v>103</v>
+      </c>
+      <c r="N8" t="s">
+        <v>99</v>
+      </c>
+      <c r="O8" t="s">
+        <v>99</v>
+      </c>
+      <c r="P8" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>100</v>
+      </c>
+      <c r="R8" t="s">
+        <v>99</v>
+      </c>
+      <c r="S8" t="s">
+        <v>101</v>
+      </c>
+      <c r="T8" t="s">
+        <v>99</v>
+      </c>
+      <c r="U8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G9" t="s">
+        <v>74</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9" t="s">
+        <v>76</v>
+      </c>
+      <c r="J9" t="s">
+        <v>77</v>
+      </c>
+      <c r="K9" t="s">
+        <v>97</v>
+      </c>
+      <c r="L9" t="s">
+        <v>97</v>
+      </c>
+      <c r="M9" t="s">
+        <v>103</v>
+      </c>
+      <c r="N9" t="s">
+        <v>99</v>
+      </c>
+      <c r="O9" t="s">
+        <v>99</v>
+      </c>
+      <c r="P9" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>100</v>
+      </c>
+      <c r="R9" t="s">
+        <v>99</v>
+      </c>
+      <c r="S9" t="s">
+        <v>101</v>
+      </c>
+      <c r="T9" t="s">
+        <v>99</v>
+      </c>
+      <c r="U9" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" t="s">
+        <v>80</v>
+      </c>
+      <c r="G10" t="s">
+        <v>81</v>
+      </c>
+      <c r="H10" t="s">
+        <v>82</v>
+      </c>
+      <c r="I10" t="s">
+        <v>83</v>
+      </c>
+      <c r="J10" t="s">
+        <v>84</v>
+      </c>
+      <c r="K10" t="s">
+        <v>97</v>
+      </c>
+      <c r="L10" t="s">
+        <v>97</v>
+      </c>
+      <c r="M10" t="s">
+        <v>103</v>
+      </c>
+      <c r="N10" t="s">
+        <v>99</v>
+      </c>
+      <c r="O10" t="s">
+        <v>99</v>
+      </c>
+      <c r="P10" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>100</v>
+      </c>
+      <c r="R10" t="s">
+        <v>99</v>
+      </c>
+      <c r="S10" t="s">
+        <v>101</v>
+      </c>
+      <c r="T10" t="s">
+        <v>99</v>
+      </c>
+      <c r="U10" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D11" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G11" t="s">
+        <v>87</v>
+      </c>
+      <c r="H11" t="s">
+        <v>88</v>
+      </c>
+      <c r="I11" t="s">
+        <v>89</v>
+      </c>
+      <c r="J11" t="s">
+        <v>90</v>
+      </c>
+      <c r="K11" t="s">
+        <v>97</v>
+      </c>
+      <c r="L11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M11" t="s">
+        <v>112</v>
+      </c>
+      <c r="N11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O11" t="s">
+        <v>99</v>
+      </c>
+      <c r="P11" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>100</v>
+      </c>
+      <c r="R11" t="s">
+        <v>99</v>
+      </c>
+      <c r="S11" t="s">
+        <v>101</v>
+      </c>
+      <c r="T11" t="s">
+        <v>99</v>
+      </c>
+      <c r="U11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D12" t="s">
+        <v>91</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" t="s">
+        <v>93</v>
+      </c>
+      <c r="I12" t="s">
+        <v>94</v>
+      </c>
+      <c r="J12" t="s">
+        <v>95</v>
+      </c>
+      <c r="K12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L12" t="s">
+        <v>97</v>
+      </c>
+      <c r="M12" t="s">
+        <v>103</v>
+      </c>
+      <c r="N12" t="s">
+        <v>99</v>
+      </c>
+      <c r="O12" t="s">
+        <v>99</v>
+      </c>
+      <c r="P12" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>100</v>
+      </c>
+      <c r="R12" t="s">
+        <v>99</v>
+      </c>
+      <c r="S12" t="s">
+        <v>101</v>
+      </c>
+      <c r="T12" t="s">
+        <v>99</v>
+      </c>
+      <c r="U12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:U13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" t="s">
+        <v>114</v>
+      </c>
+      <c r="L2" t="s">
+        <v>97</v>
+      </c>
+      <c r="M2" t="s">
+        <v>115</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2" t="s">
+        <v>116</v>
+      </c>
+      <c r="P2">
+        <v>5</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>117</v>
+      </c>
+      <c r="R2" t="s">
+        <v>118</v>
+      </c>
+      <c r="S2" t="s">
+        <v>118</v>
+      </c>
+      <c r="U2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" t="s">
+        <v>120</v>
+      </c>
+      <c r="L3" t="s">
+        <v>97</v>
+      </c>
+      <c r="M3" t="s">
+        <v>121</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3" t="s">
+        <v>122</v>
+      </c>
+      <c r="P3">
+        <v>3</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>123</v>
+      </c>
+      <c r="R3" t="s">
+        <v>124</v>
+      </c>
+      <c r="S3" t="s">
+        <v>125</v>
+      </c>
+      <c r="U3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K4" t="s">
+        <v>126</v>
+      </c>
+      <c r="L4" t="s">
+        <v>127</v>
+      </c>
+      <c r="M4" t="s">
+        <v>128</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4" t="s">
+        <v>108</v>
+      </c>
+      <c r="P4">
+        <v>3</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>129</v>
+      </c>
+      <c r="R4" t="s">
+        <v>130</v>
+      </c>
+      <c r="S4" t="s">
+        <v>125</v>
+      </c>
+      <c r="U4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>131</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" t="s">
+        <v>132</v>
+      </c>
+      <c r="H5" t="s">
+        <v>133</v>
+      </c>
+      <c r="I5" t="s">
+        <v>134</v>
+      </c>
+      <c r="J5" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L5" t="s">
+        <v>97</v>
+      </c>
+      <c r="M5" t="s">
+        <v>128</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5" t="s">
+        <v>122</v>
+      </c>
+      <c r="P5">
+        <v>4</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>135</v>
+      </c>
+      <c r="R5" t="s">
+        <v>118</v>
+      </c>
+      <c r="S5" t="s">
+        <v>118</v>
+      </c>
+      <c r="U5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" t="s">
+        <v>55</v>
+      </c>
+      <c r="J6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K6" t="s">
+        <v>136</v>
+      </c>
+      <c r="L6" t="s">
+        <v>97</v>
+      </c>
+      <c r="M6" t="s">
+        <v>137</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6" t="s">
+        <v>122</v>
+      </c>
+      <c r="P6">
+        <v>4</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>138</v>
+      </c>
+      <c r="R6" t="s">
+        <v>118</v>
+      </c>
+      <c r="S6" t="s">
+        <v>139</v>
+      </c>
+      <c r="U6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" t="s">
+        <v>62</v>
+      </c>
+      <c r="J7" t="s">
+        <v>63</v>
+      </c>
+      <c r="K7" t="s">
+        <v>140</v>
+      </c>
+      <c r="L7" t="s">
+        <v>141</v>
+      </c>
+      <c r="M7" t="s">
+        <v>128</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7" t="s">
+        <v>116</v>
+      </c>
+      <c r="P7">
+        <v>4</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>117</v>
+      </c>
+      <c r="R7" t="s">
+        <v>118</v>
+      </c>
+      <c r="S7" t="s">
+        <v>118</v>
+      </c>
+      <c r="U7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" t="s">
+        <v>67</v>
+      </c>
+      <c r="H8" t="s">
+        <v>68</v>
+      </c>
+      <c r="I8" t="s">
+        <v>69</v>
+      </c>
+      <c r="J8" t="s">
+        <v>70</v>
+      </c>
+      <c r="K8" t="s">
+        <v>140</v>
+      </c>
+      <c r="L8" t="s">
+        <v>141</v>
+      </c>
+      <c r="M8" t="s">
+        <v>121</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8" t="s">
+        <v>116</v>
+      </c>
+      <c r="P8">
+        <v>3</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>142</v>
+      </c>
+      <c r="R8" t="s">
+        <v>143</v>
+      </c>
+      <c r="S8" t="s">
+        <v>118</v>
+      </c>
+      <c r="U8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G9" t="s">
+        <v>74</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9" t="s">
+        <v>76</v>
+      </c>
+      <c r="J9" t="s">
+        <v>77</v>
+      </c>
+      <c r="K9" t="s">
+        <v>140</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="M9" t="s">
+        <v>128</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9" t="s">
+        <v>116</v>
+      </c>
+      <c r="P9">
+        <v>5</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>117</v>
+      </c>
+      <c r="R9" t="s">
+        <v>118</v>
+      </c>
+      <c r="S9" t="s">
+        <v>118</v>
+      </c>
+      <c r="U9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="M13" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Se elimian los Seed iniciales, se ajustan las guias de usuario
</commit_message>
<xml_diff>
--- a/docs/pruebas_usabilidad_ieee29119-11.xlsx
+++ b/docs/pruebas_usabilidad_ieee29119-11.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13392" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13390" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="plantilla_registro_pruebas_usab" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="146">
   <si>
     <t>ID Registro</t>
   </si>
@@ -453,6 +453,12 @@
   </si>
   <si>
     <t>Baja</t>
+  </si>
+  <si>
+    <t>30seg</t>
+  </si>
+  <si>
+    <t>40seg</t>
   </si>
 </sst>
 </file>
@@ -792,31 +798,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="54.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="97.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="60.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="27.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="31.77734375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="54.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="97.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="60.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.6328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="20.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -881,7 +887,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -910,7 +916,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -939,7 +945,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -968,7 +974,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -997,7 +1003,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -1026,7 +1032,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -1055,7 +1061,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>64</v>
       </c>
@@ -1084,7 +1090,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -1113,10 +1119,10 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -1145,7 +1151,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>78</v>
       </c>
@@ -1174,7 +1180,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>85</v>
       </c>
@@ -1203,7 +1209,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
     </row>
   </sheetData>
@@ -1215,9 +1221,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1282,7 +1288,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1344,7 +1350,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -1406,7 +1412,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -1468,7 +1474,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1530,7 +1536,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -1592,7 +1598,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -1654,7 +1660,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>64</v>
       </c>
@@ -1716,7 +1722,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -1778,7 +1784,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>96</v>
       </c>
@@ -1840,7 +1846,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>78</v>
       </c>
@@ -1902,7 +1908,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -1973,9 +1979,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="7" max="7" width="24.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2040,7 +2049,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -2099,7 +2108,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -2158,7 +2167,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -2217,7 +2226,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -2276,7 +2285,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -2335,7 +2344,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -2394,7 +2403,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>64</v>
       </c>
@@ -2453,7 +2462,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -2512,7 +2521,184 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" t="s">
+        <v>80</v>
+      </c>
+      <c r="G10" t="s">
+        <v>81</v>
+      </c>
+      <c r="H10" t="s">
+        <v>82</v>
+      </c>
+      <c r="I10" t="s">
+        <v>83</v>
+      </c>
+      <c r="J10" t="s">
+        <v>84</v>
+      </c>
+      <c r="K10" t="s">
+        <v>97</v>
+      </c>
+      <c r="L10" t="s">
+        <v>97</v>
+      </c>
+      <c r="M10" t="s">
+        <v>144</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10" t="s">
+        <v>116</v>
+      </c>
+      <c r="P10">
+        <v>5</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>117</v>
+      </c>
+      <c r="R10" t="s">
+        <v>118</v>
+      </c>
+      <c r="S10" t="s">
+        <v>118</v>
+      </c>
+      <c r="U10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G11" t="s">
+        <v>87</v>
+      </c>
+      <c r="H11" t="s">
+        <v>88</v>
+      </c>
+      <c r="I11" t="s">
+        <v>89</v>
+      </c>
+      <c r="J11" t="s">
+        <v>90</v>
+      </c>
+      <c r="K11" t="s">
+        <v>97</v>
+      </c>
+      <c r="L11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M11" t="s">
+        <v>145</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11" t="s">
+        <v>116</v>
+      </c>
+      <c r="P11">
+        <v>5</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>117</v>
+      </c>
+      <c r="R11" t="s">
+        <v>118</v>
+      </c>
+      <c r="S11" t="s">
+        <v>118</v>
+      </c>
+      <c r="U11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>91</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" t="s">
+        <v>93</v>
+      </c>
+      <c r="I12" t="s">
+        <v>94</v>
+      </c>
+      <c r="J12" t="s">
+        <v>95</v>
+      </c>
+      <c r="K12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L12" t="s">
+        <v>97</v>
+      </c>
+      <c r="M12" t="s">
+        <v>144</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12" t="s">
+        <v>116</v>
+      </c>
+      <c r="P12">
+        <v>5</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>117</v>
+      </c>
+      <c r="R12" t="s">
+        <v>118</v>
+      </c>
+      <c r="S12" t="s">
+        <v>118</v>
+      </c>
+      <c r="U12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
       <c r="M13" s="2"/>
     </row>
   </sheetData>

</xml_diff>